<commit_message>
feat: update data Juni 2026, retrain forecast, redeploy HF Space
- Data inflasi MoM Juni 2026: +0.44% (BPS)
- IHK Juni 2026: 124.06 (diperhitungkan dari IHK Mei + MoM)
- BI Rate Juni 2026: 3.34% (BI)
- USD/IDR Juni 2026: rata-rata ~17,898 (Investing.com + Yahoo Finance)
- Brent Oil Juni 2026: 72.92 USD/barel (Yahoo Finance BZ=F)
- WTI Juni 2026: 69.50 USD/barel (Yahoo Finance CL=F)
- DXY Juni 2026: 101.19 (Yahoo Finance DX-Y.NYB)
- Gold Juni 2026: 4,022.90 USD/oz (Yahoo Finance GC=F)
- FedRate Juni 2026: 3.63% (Fed tidak berubah)
- Retrain inflation_multihorizon: prediksi Juli 2026 +0.36% MoM (ARIMA)
- 28/28 Django tests passed
- Tambah Dockerfile, hf-space/, scripts/deploy_hf_space.ps1, DEPLOY_HF_SPACES.md
- Tambah update_june_international.py untuk update data eksogen via yfinance
</commit_message>
<xml_diff>
--- a/datasets/BI Rate (Data Inflasi)/Data Inflasi.xlsx
+++ b/datasets/BI Rate (Data Inflasi)/Data Inflasi.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="522">
   <si>
     <t>Data Inflasi</t>
   </si>
@@ -23,6 +23,30 @@
     <t>Periode</t>
   </si>
   <si>
+    <t>Juni 2026</t>
+  </si>
+  <si>
+    <t>3.34 %</t>
+  </si>
+  <si>
+    <t>Mei 2026</t>
+  </si>
+  <si>
+    <t>3.08 %</t>
+  </si>
+  <si>
+    <t>April 2026</t>
+  </si>
+  <si>
+    <t>2.42 %</t>
+  </si>
+  <si>
+    <t>Maret 2026</t>
+  </si>
+  <si>
+    <t>3.48 %</t>
+  </si>
+  <si>
     <t>Februari 2026</t>
   </si>
   <si>
@@ -209,9 +233,6 @@
     <t>Juli 2023</t>
   </si>
   <si>
-    <t>3.08 %</t>
-  </si>
-  <si>
     <t>Juni 2023</t>
   </si>
   <si>
@@ -1425,6 +1446,138 @@
   </si>
   <si>
     <t>Januari 2005</t>
+  </si>
+  <si>
+    <t>Desember 2004</t>
+  </si>
+  <si>
+    <t>6.4 %</t>
+  </si>
+  <si>
+    <t>November 2004</t>
+  </si>
+  <si>
+    <t>6.18 %</t>
+  </si>
+  <si>
+    <t>Oktober 2004</t>
+  </si>
+  <si>
+    <t>September 2004</t>
+  </si>
+  <si>
+    <t>6.27 %</t>
+  </si>
+  <si>
+    <t>Agustus 2004</t>
+  </si>
+  <si>
+    <t>6.67 %</t>
+  </si>
+  <si>
+    <t>Juli 2004</t>
+  </si>
+  <si>
+    <t>7.2 %</t>
+  </si>
+  <si>
+    <t>Juni 2004</t>
+  </si>
+  <si>
+    <t>Mei 2004</t>
+  </si>
+  <si>
+    <t>6.47 %</t>
+  </si>
+  <si>
+    <t>April 2004</t>
+  </si>
+  <si>
+    <t>5.92 %</t>
+  </si>
+  <si>
+    <t>Maret 2004</t>
+  </si>
+  <si>
+    <t>5.11 %</t>
+  </si>
+  <si>
+    <t>Februari 2004</t>
+  </si>
+  <si>
+    <t>4.6 %</t>
+  </si>
+  <si>
+    <t>Januari 2004</t>
+  </si>
+  <si>
+    <t>4.82 %</t>
+  </si>
+  <si>
+    <t>Desember 2003</t>
+  </si>
+  <si>
+    <t>5.16 %</t>
+  </si>
+  <si>
+    <t>November 2003</t>
+  </si>
+  <si>
+    <t>5.53 %</t>
+  </si>
+  <si>
+    <t>Oktober 2003</t>
+  </si>
+  <si>
+    <t>6.48 %</t>
+  </si>
+  <si>
+    <t>September 2003</t>
+  </si>
+  <si>
+    <t>Agustus 2003</t>
+  </si>
+  <si>
+    <t>Juli 2003</t>
+  </si>
+  <si>
+    <t>Juni 2003</t>
+  </si>
+  <si>
+    <t>6.98 %</t>
+  </si>
+  <si>
+    <t>Mei 2003</t>
+  </si>
+  <si>
+    <t>April 2003</t>
+  </si>
+  <si>
+    <t>7.62 %</t>
+  </si>
+  <si>
+    <t>Maret 2003</t>
+  </si>
+  <si>
+    <t>7.17 %</t>
+  </si>
+  <si>
+    <t>Februari 2003</t>
+  </si>
+  <si>
+    <t>7.6 %</t>
+  </si>
+  <si>
+    <t>Januari 2003</t>
+  </si>
+  <si>
+    <t>8.68 %</t>
+  </si>
+  <si>
+    <t>Desember 2002</t>
+  </si>
+  <si>
+    <t>0 %</t>
   </si>
 </sst>
 </file>
@@ -1500,7 +1653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="xr">
-  <dimension ref="A3:D259"/>
+  <dimension ref="A3:D288"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -1833,7 +1986,7 @@
         <v>57</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>12</v>
+        <v>58</v>
       </c>
     </row>
     <row r="34">
@@ -1841,10 +1994,10 @@
         <v>29</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35">
@@ -1852,10 +2005,10 @@
         <v>30</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36">
@@ -1863,10 +2016,10 @@
         <v>31</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37">
@@ -1874,10 +2027,10 @@
         <v>32</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38">
@@ -1921,7 +2074,7 @@
         <v>72</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>73</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42">
@@ -1929,10 +2082,10 @@
         <v>37</v>
       </c>
       <c r="B42" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C42" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="43">
@@ -1940,10 +2093,10 @@
         <v>38</v>
       </c>
       <c r="B43" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C43" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="44">
@@ -1951,10 +2104,10 @@
         <v>39</v>
       </c>
       <c r="B44" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C44" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="45">
@@ -1962,10 +2115,10 @@
         <v>40</v>
       </c>
       <c r="B45" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C45" s="3" t="s">
         <v>80</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="46">
@@ -1973,10 +2126,10 @@
         <v>41</v>
       </c>
       <c r="B46" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C46" s="3" t="s">
         <v>82</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="47">
@@ -1984,10 +2137,10 @@
         <v>42</v>
       </c>
       <c r="B47" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C47" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="48">
@@ -1995,10 +2148,10 @@
         <v>43</v>
       </c>
       <c r="B48" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C48" s="3" t="s">
         <v>86</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="49">
@@ -2006,10 +2159,10 @@
         <v>44</v>
       </c>
       <c r="B49" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C49" s="3" t="s">
         <v>88</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="50">
@@ -2017,10 +2170,10 @@
         <v>45</v>
       </c>
       <c r="B50" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C50" s="3" t="s">
         <v>90</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="51">
@@ -2028,10 +2181,10 @@
         <v>46</v>
       </c>
       <c r="B51" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C51" s="3" t="s">
         <v>92</v>
-      </c>
-      <c r="C51" s="3" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="52">
@@ -2075,7 +2228,7 @@
         <v>99</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>100</v>
+        <v>14</v>
       </c>
     </row>
     <row r="56">
@@ -2083,10 +2236,10 @@
         <v>51</v>
       </c>
       <c r="B56" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C56" s="3" t="s">
         <v>101</v>
-      </c>
-      <c r="C56" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="57">
@@ -2119,7 +2272,7 @@
         <v>106</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>22</v>
+        <v>107</v>
       </c>
     </row>
     <row r="60">
@@ -2127,10 +2280,10 @@
         <v>55</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>108</v>
+        <v>28</v>
       </c>
     </row>
     <row r="61">
@@ -2163,7 +2316,7 @@
         <v>113</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>114</v>
+        <v>30</v>
       </c>
     </row>
     <row r="64">
@@ -2171,10 +2324,10 @@
         <v>59</v>
       </c>
       <c r="B64" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C64" s="3" t="s">
         <v>115</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="65">
@@ -2182,10 +2335,10 @@
         <v>60</v>
       </c>
       <c r="B65" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C65" s="3" t="s">
         <v>117</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="66">
@@ -2193,10 +2346,10 @@
         <v>61</v>
       </c>
       <c r="B66" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C66" s="3" t="s">
         <v>119</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="67">
@@ -2204,10 +2357,10 @@
         <v>62</v>
       </c>
       <c r="B67" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C67" s="3" t="s">
         <v>121</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="68">
@@ -2218,7 +2371,7 @@
         <v>122</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
     <row r="69">
@@ -2226,10 +2379,10 @@
         <v>64</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
     </row>
     <row r="70">
@@ -2237,10 +2390,10 @@
         <v>65</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="71">
@@ -2248,10 +2401,10 @@
         <v>66</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>116</v>
+        <v>42</v>
       </c>
     </row>
     <row r="72">
@@ -2259,10 +2412,10 @@
         <v>67</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
     </row>
     <row r="73">
@@ -2270,10 +2423,10 @@
         <v>68</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
     </row>
     <row r="74">
@@ -2295,7 +2448,7 @@
         <v>133</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
     </row>
     <row r="76">
@@ -2303,10 +2456,10 @@
         <v>71</v>
       </c>
       <c r="B76" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C76" s="3" t="s">
         <v>135</v>
-      </c>
-      <c r="C76" s="3" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="77">
@@ -2314,10 +2467,10 @@
         <v>72</v>
       </c>
       <c r="B77" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C77" s="3" t="s">
         <v>137</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="78">
@@ -2325,10 +2478,10 @@
         <v>73</v>
       </c>
       <c r="B78" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C78" s="3" t="s">
         <v>139</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="79">
@@ -2336,10 +2489,10 @@
         <v>74</v>
       </c>
       <c r="B79" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C79" s="3" t="s">
         <v>141</v>
-      </c>
-      <c r="C79" s="3" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="80">
@@ -2347,10 +2500,10 @@
         <v>75</v>
       </c>
       <c r="B80" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C80" s="3" t="s">
         <v>143</v>
-      </c>
-      <c r="C80" s="3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="81">
@@ -2361,7 +2514,7 @@
         <v>144</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>48</v>
+        <v>145</v>
       </c>
     </row>
     <row r="82">
@@ -2369,10 +2522,10 @@
         <v>77</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="83">
@@ -2380,10 +2533,10 @@
         <v>78</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="84">
@@ -2391,10 +2544,10 @@
         <v>79</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>150</v>
+        <v>18</v>
       </c>
     </row>
     <row r="85">
@@ -2405,7 +2558,7 @@
         <v>151</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>152</v>
+        <v>56</v>
       </c>
     </row>
     <row r="86">
@@ -2413,10 +2566,10 @@
         <v>81</v>
       </c>
       <c r="B86" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C86" s="3" t="s">
         <v>153</v>
-      </c>
-      <c r="C86" s="3" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="87">
@@ -2424,10 +2577,10 @@
         <v>82</v>
       </c>
       <c r="B87" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C87" s="3" t="s">
         <v>155</v>
-      </c>
-      <c r="C87" s="3" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="88">
@@ -2460,7 +2613,7 @@
         <v>160</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>54</v>
+        <v>161</v>
       </c>
     </row>
     <row r="91">
@@ -2468,10 +2621,10 @@
         <v>86</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="92">
@@ -2482,7 +2635,7 @@
         <v>163</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>146</v>
+        <v>164</v>
       </c>
     </row>
     <row r="93">
@@ -2490,10 +2643,10 @@
         <v>88</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="94">
@@ -2501,10 +2654,10 @@
         <v>89</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>167</v>
+        <v>62</v>
       </c>
     </row>
     <row r="95">
@@ -2526,7 +2679,7 @@
         <v>170</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
     </row>
     <row r="97">
@@ -2534,10 +2687,10 @@
         <v>92</v>
       </c>
       <c r="B97" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C97" s="3" t="s">
         <v>172</v>
-      </c>
-      <c r="C97" s="3" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="98">
@@ -2545,10 +2698,10 @@
         <v>93</v>
       </c>
       <c r="B98" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="C98" s="3" t="s">
         <v>174</v>
-      </c>
-      <c r="C98" s="3" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="99">
@@ -2556,10 +2709,10 @@
         <v>94</v>
       </c>
       <c r="B99" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C99" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="C99" s="3" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="100">
@@ -2592,7 +2745,7 @@
         <v>181</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
     </row>
     <row r="103">
@@ -2600,10 +2753,10 @@
         <v>98</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
     </row>
     <row r="104">
@@ -2636,7 +2789,7 @@
         <v>188</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="107">
@@ -2644,10 +2797,10 @@
         <v>102</v>
       </c>
       <c r="B107" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C107" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="C107" s="3" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="108">
@@ -2655,10 +2808,10 @@
         <v>103</v>
       </c>
       <c r="B108" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="C108" s="3" t="s">
         <v>192</v>
-      </c>
-      <c r="C108" s="3" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="109">
@@ -2666,10 +2819,10 @@
         <v>104</v>
       </c>
       <c r="B109" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="C109" s="3" t="s">
         <v>194</v>
-      </c>
-      <c r="C109" s="3" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="110">
@@ -2677,10 +2830,10 @@
         <v>105</v>
       </c>
       <c r="B110" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="C110" s="3" t="s">
         <v>196</v>
-      </c>
-      <c r="C110" s="3" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="111">
@@ -2688,10 +2841,10 @@
         <v>106</v>
       </c>
       <c r="B111" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="C111" s="3" t="s">
         <v>198</v>
-      </c>
-      <c r="C111" s="3" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="112">
@@ -2713,7 +2866,7 @@
         <v>201</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>185</v>
+        <v>202</v>
       </c>
     </row>
     <row r="114">
@@ -2721,10 +2874,10 @@
         <v>109</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="115">
@@ -2732,10 +2885,10 @@
         <v>110</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>150</v>
+        <v>78</v>
       </c>
     </row>
     <row r="116">
@@ -2743,10 +2896,10 @@
         <v>111</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="117">
@@ -2754,10 +2907,10 @@
         <v>112</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="118">
@@ -2765,10 +2918,10 @@
         <v>113</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="119">
@@ -2776,10 +2929,10 @@
         <v>114</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>211</v>
+        <v>157</v>
       </c>
     </row>
     <row r="120">
@@ -2801,7 +2954,7 @@
         <v>214</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>215</v>
+        <v>196</v>
       </c>
     </row>
     <row r="122">
@@ -2809,10 +2962,10 @@
         <v>117</v>
       </c>
       <c r="B122" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="C122" s="3" t="s">
         <v>216</v>
-      </c>
-      <c r="C122" s="3" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="123">
@@ -2820,10 +2973,10 @@
         <v>118</v>
       </c>
       <c r="B123" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="C123" s="3" t="s">
         <v>218</v>
-      </c>
-      <c r="C123" s="3" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="124">
@@ -2831,10 +2984,10 @@
         <v>119</v>
       </c>
       <c r="B124" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="C124" s="3" t="s">
         <v>220</v>
-      </c>
-      <c r="C124" s="3" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="125">
@@ -2842,10 +2995,10 @@
         <v>120</v>
       </c>
       <c r="B125" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="C125" s="3" t="s">
         <v>222</v>
-      </c>
-      <c r="C125" s="3" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="126">
@@ -2853,10 +3006,10 @@
         <v>121</v>
       </c>
       <c r="B126" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="C126" s="3" t="s">
         <v>224</v>
-      </c>
-      <c r="C126" s="3" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="127">
@@ -2864,10 +3017,10 @@
         <v>122</v>
       </c>
       <c r="B127" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C127" s="3" t="s">
         <v>226</v>
-      </c>
-      <c r="C127" s="3" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="128">
@@ -2875,10 +3028,10 @@
         <v>123</v>
       </c>
       <c r="B128" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="C128" s="3" t="s">
         <v>228</v>
-      </c>
-      <c r="C128" s="3" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="129">
@@ -2886,10 +3039,10 @@
         <v>124</v>
       </c>
       <c r="B129" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="C129" s="3" t="s">
         <v>230</v>
-      </c>
-      <c r="C129" s="3" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="130">
@@ -2897,10 +3050,10 @@
         <v>125</v>
       </c>
       <c r="B130" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="C130" s="3" t="s">
         <v>232</v>
-      </c>
-      <c r="C130" s="3" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="131">
@@ -2908,10 +3061,10 @@
         <v>126</v>
       </c>
       <c r="B131" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C131" s="3" t="s">
         <v>234</v>
-      </c>
-      <c r="C131" s="3" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="132">
@@ -2919,10 +3072,10 @@
         <v>127</v>
       </c>
       <c r="B132" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="C132" s="3" t="s">
         <v>236</v>
-      </c>
-      <c r="C132" s="3" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="133">
@@ -2930,10 +3083,10 @@
         <v>128</v>
       </c>
       <c r="B133" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="C133" s="3" t="s">
         <v>238</v>
-      </c>
-      <c r="C133" s="3" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="134">
@@ -2941,10 +3094,10 @@
         <v>129</v>
       </c>
       <c r="B134" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C134" s="3" t="s">
         <v>240</v>
-      </c>
-      <c r="C134" s="3" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="135">
@@ -2988,7 +3141,7 @@
         <v>247</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="139">
@@ -2996,10 +3149,10 @@
         <v>134</v>
       </c>
       <c r="B139" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="C139" s="3" t="s">
         <v>249</v>
-      </c>
-      <c r="C139" s="3" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="140">
@@ -3007,10 +3160,10 @@
         <v>135</v>
       </c>
       <c r="B140" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="C140" s="3" t="s">
         <v>251</v>
-      </c>
-      <c r="C140" s="3" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="141">
@@ -3018,10 +3171,10 @@
         <v>136</v>
       </c>
       <c r="B141" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="C141" s="3" t="s">
         <v>253</v>
-      </c>
-      <c r="C141" s="3" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="142">
@@ -3029,10 +3182,10 @@
         <v>137</v>
       </c>
       <c r="B142" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="C142" s="3" t="s">
         <v>255</v>
-      </c>
-      <c r="C142" s="3" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="143">
@@ -3040,10 +3193,10 @@
         <v>138</v>
       </c>
       <c r="B143" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="C143" s="3" t="s">
         <v>257</v>
-      </c>
-      <c r="C143" s="3" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="144">
@@ -3051,10 +3204,10 @@
         <v>139</v>
       </c>
       <c r="B144" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="C144" s="3" t="s">
         <v>259</v>
-      </c>
-      <c r="C144" s="3" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="145">
@@ -3062,10 +3215,10 @@
         <v>140</v>
       </c>
       <c r="B145" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="C145" s="3" t="s">
         <v>261</v>
-      </c>
-      <c r="C145" s="3" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="146">
@@ -3153,7 +3306,7 @@
         <v>275</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
     </row>
     <row r="154">
@@ -3161,10 +3314,10 @@
         <v>149</v>
       </c>
       <c r="B154" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="C154" s="3" t="s">
         <v>277</v>
-      </c>
-      <c r="C154" s="3" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="155">
@@ -3172,10 +3325,10 @@
         <v>150</v>
       </c>
       <c r="B155" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="C155" s="3" t="s">
         <v>279</v>
-      </c>
-      <c r="C155" s="3" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="156">
@@ -3183,10 +3336,10 @@
         <v>151</v>
       </c>
       <c r="B156" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="C156" s="3" t="s">
         <v>281</v>
-      </c>
-      <c r="C156" s="3" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="157">
@@ -3194,10 +3347,10 @@
         <v>152</v>
       </c>
       <c r="B157" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="C157" s="3" t="s">
         <v>283</v>
-      </c>
-      <c r="C157" s="3" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="158">
@@ -3205,10 +3358,10 @@
         <v>153</v>
       </c>
       <c r="B158" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="C158" s="3" t="s">
         <v>285</v>
-      </c>
-      <c r="C158" s="3" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="159">
@@ -3216,10 +3369,10 @@
         <v>154</v>
       </c>
       <c r="B159" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="C159" s="3" t="s">
         <v>287</v>
-      </c>
-      <c r="C159" s="3" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="160">
@@ -3241,7 +3394,7 @@
         <v>290</v>
       </c>
       <c r="C161" s="3" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
     </row>
     <row r="162">
@@ -3249,10 +3402,10 @@
         <v>157</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C162" s="3" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="163">
@@ -3260,10 +3413,10 @@
         <v>158</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C163" s="3" t="s">
-        <v>294</v>
+        <v>82</v>
       </c>
     </row>
     <row r="164">
@@ -3285,7 +3438,7 @@
         <v>297</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
     </row>
     <row r="166">
@@ -3293,10 +3446,10 @@
         <v>161</v>
       </c>
       <c r="B166" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="C166" s="3" t="s">
         <v>299</v>
-      </c>
-      <c r="C166" s="3" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="167">
@@ -3304,10 +3457,10 @@
         <v>162</v>
       </c>
       <c r="B167" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="C167" s="3" t="s">
         <v>301</v>
-      </c>
-      <c r="C167" s="3" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="168">
@@ -3315,10 +3468,10 @@
         <v>163</v>
       </c>
       <c r="B168" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="C168" s="3" t="s">
         <v>303</v>
-      </c>
-      <c r="C168" s="3" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="169">
@@ -3326,10 +3479,10 @@
         <v>164</v>
       </c>
       <c r="B169" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="C169" s="3" t="s">
         <v>305</v>
-      </c>
-      <c r="C169" s="3" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="170">
@@ -3337,10 +3490,10 @@
         <v>165</v>
       </c>
       <c r="B170" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="C170" s="3" t="s">
         <v>307</v>
-      </c>
-      <c r="C170" s="3" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="171">
@@ -3351,7 +3504,7 @@
         <v>308</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>223</v>
+        <v>309</v>
       </c>
     </row>
     <row r="172">
@@ -3359,10 +3512,10 @@
         <v>167</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C172" s="3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="173">
@@ -3370,10 +3523,10 @@
         <v>168</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C173" s="3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="174">
@@ -3381,10 +3534,10 @@
         <v>169</v>
       </c>
       <c r="B174" s="3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C174" s="3" t="s">
-        <v>314</v>
+        <v>265</v>
       </c>
     </row>
     <row r="175">
@@ -3395,7 +3548,7 @@
         <v>315</v>
       </c>
       <c r="C175" s="3" t="s">
-        <v>316</v>
+        <v>230</v>
       </c>
     </row>
     <row r="176">
@@ -3403,10 +3556,10 @@
         <v>171</v>
       </c>
       <c r="B176" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="C176" s="3" t="s">
         <v>317</v>
-      </c>
-      <c r="C176" s="3" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="177">
@@ -3414,10 +3567,10 @@
         <v>172</v>
       </c>
       <c r="B177" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="C177" s="3" t="s">
         <v>319</v>
-      </c>
-      <c r="C177" s="3" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="178">
@@ -3425,10 +3578,10 @@
         <v>173</v>
       </c>
       <c r="B178" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="C178" s="3" t="s">
         <v>321</v>
-      </c>
-      <c r="C178" s="3" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="179">
@@ -3439,7 +3592,7 @@
         <v>322</v>
       </c>
       <c r="C179" s="3" t="s">
-        <v>300</v>
+        <v>323</v>
       </c>
     </row>
     <row r="180">
@@ -3447,10 +3600,10 @@
         <v>175</v>
       </c>
       <c r="B180" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C180" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="181">
@@ -3458,10 +3611,10 @@
         <v>176</v>
       </c>
       <c r="B181" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C181" s="3" t="s">
-        <v>300</v>
+        <v>327</v>
       </c>
     </row>
     <row r="182">
@@ -3469,10 +3622,10 @@
         <v>177</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C182" s="3" t="s">
-        <v>327</v>
+        <v>232</v>
       </c>
     </row>
     <row r="183">
@@ -3480,10 +3633,10 @@
         <v>178</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C183" s="3" t="s">
-        <v>329</v>
+        <v>307</v>
       </c>
     </row>
     <row r="184">
@@ -3505,7 +3658,7 @@
         <v>332</v>
       </c>
       <c r="C185" s="3" t="s">
-        <v>333</v>
+        <v>307</v>
       </c>
     </row>
     <row r="186">
@@ -3513,10 +3666,10 @@
         <v>181</v>
       </c>
       <c r="B186" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C186" s="3" t="s">
         <v>334</v>
-      </c>
-      <c r="C186" s="3" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="187">
@@ -3524,10 +3677,10 @@
         <v>182</v>
       </c>
       <c r="B187" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="C187" s="3" t="s">
         <v>336</v>
-      </c>
-      <c r="C187" s="3" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="188">
@@ -3535,10 +3688,10 @@
         <v>183</v>
       </c>
       <c r="B188" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="C188" s="3" t="s">
         <v>338</v>
-      </c>
-      <c r="C188" s="3" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="189">
@@ -3582,7 +3735,7 @@
         <v>345</v>
       </c>
       <c r="C192" s="3" t="s">
-        <v>346</v>
+        <v>257</v>
       </c>
     </row>
     <row r="193">
@@ -3590,10 +3743,10 @@
         <v>188</v>
       </c>
       <c r="B193" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="C193" s="3" t="s">
         <v>347</v>
-      </c>
-      <c r="C193" s="3" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="194">
@@ -3601,10 +3754,10 @@
         <v>189</v>
       </c>
       <c r="B194" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="C194" s="3" t="s">
         <v>349</v>
-      </c>
-      <c r="C194" s="3" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="195">
@@ -3612,10 +3765,10 @@
         <v>190</v>
       </c>
       <c r="B195" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="C195" s="3" t="s">
         <v>351</v>
-      </c>
-      <c r="C195" s="3" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="196">
@@ -3623,10 +3776,10 @@
         <v>191</v>
       </c>
       <c r="B196" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="C196" s="3" t="s">
         <v>353</v>
-      </c>
-      <c r="C196" s="3" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="197">
@@ -3634,10 +3787,10 @@
         <v>192</v>
       </c>
       <c r="B197" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="C197" s="3" t="s">
         <v>355</v>
-      </c>
-      <c r="C197" s="3" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="198">
@@ -3645,10 +3798,10 @@
         <v>193</v>
       </c>
       <c r="B198" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="C198" s="3" t="s">
         <v>357</v>
-      </c>
-      <c r="C198" s="3" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="199">
@@ -3656,10 +3809,10 @@
         <v>194</v>
       </c>
       <c r="B199" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="C199" s="3" t="s">
         <v>359</v>
-      </c>
-      <c r="C199" s="3" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="200">
@@ -3692,7 +3845,7 @@
         <v>364</v>
       </c>
       <c r="C202" s="3" t="s">
-        <v>54</v>
+        <v>365</v>
       </c>
     </row>
     <row r="203">
@@ -3700,10 +3853,10 @@
         <v>198</v>
       </c>
       <c r="B203" s="3" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C203" s="3" t="s">
-        <v>157</v>
+        <v>198</v>
       </c>
     </row>
     <row r="204">
@@ -3711,10 +3864,10 @@
         <v>199</v>
       </c>
       <c r="B204" s="3" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C204" s="3" t="s">
-        <v>52</v>
+        <v>368</v>
       </c>
     </row>
     <row r="205">
@@ -3722,10 +3875,10 @@
         <v>200</v>
       </c>
       <c r="B205" s="3" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C205" s="3" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="206">
@@ -3733,10 +3886,10 @@
         <v>201</v>
       </c>
       <c r="B206" s="3" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C206" s="3" t="s">
-        <v>316</v>
+        <v>62</v>
       </c>
     </row>
     <row r="207">
@@ -3744,10 +3897,10 @@
         <v>202</v>
       </c>
       <c r="B207" s="3" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="C207" s="3" t="s">
-        <v>371</v>
+        <v>164</v>
       </c>
     </row>
     <row r="208">
@@ -3755,10 +3908,10 @@
         <v>203</v>
       </c>
       <c r="B208" s="3" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C208" s="3" t="s">
-        <v>373</v>
+        <v>60</v>
       </c>
     </row>
     <row r="209">
@@ -3780,7 +3933,7 @@
         <v>376</v>
       </c>
       <c r="C210" s="3" t="s">
-        <v>377</v>
+        <v>323</v>
       </c>
     </row>
     <row r="211">
@@ -3788,10 +3941,10 @@
         <v>206</v>
       </c>
       <c r="B211" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="C211" s="3" t="s">
         <v>378</v>
-      </c>
-      <c r="C211" s="3" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="212">
@@ -3799,10 +3952,10 @@
         <v>207</v>
       </c>
       <c r="B212" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="C212" s="3" t="s">
         <v>380</v>
-      </c>
-      <c r="C212" s="3" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="213">
@@ -3810,10 +3963,10 @@
         <v>208</v>
       </c>
       <c r="B213" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="C213" s="3" t="s">
         <v>382</v>
-      </c>
-      <c r="C213" s="3" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="214">
@@ -3821,10 +3974,10 @@
         <v>209</v>
       </c>
       <c r="B214" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="C214" s="3" t="s">
         <v>384</v>
-      </c>
-      <c r="C214" s="3" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="215">
@@ -3832,10 +3985,10 @@
         <v>210</v>
       </c>
       <c r="B215" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="C215" s="3" t="s">
         <v>386</v>
-      </c>
-      <c r="C215" s="3" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="216">
@@ -3843,10 +3996,10 @@
         <v>211</v>
       </c>
       <c r="B216" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="C216" s="3" t="s">
         <v>388</v>
-      </c>
-      <c r="C216" s="3" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="217">
@@ -3854,10 +4007,10 @@
         <v>212</v>
       </c>
       <c r="B217" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C217" s="3" t="s">
         <v>390</v>
-      </c>
-      <c r="C217" s="3" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="218">
@@ -3865,10 +4018,10 @@
         <v>213</v>
       </c>
       <c r="B218" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="C218" s="3" t="s">
         <v>392</v>
-      </c>
-      <c r="C218" s="3" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="219">
@@ -3876,10 +4029,10 @@
         <v>214</v>
       </c>
       <c r="B219" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C219" s="3" t="s">
         <v>394</v>
-      </c>
-      <c r="C219" s="3" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="220">
@@ -3887,10 +4040,10 @@
         <v>215</v>
       </c>
       <c r="B220" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="C220" s="3" t="s">
         <v>396</v>
-      </c>
-      <c r="C220" s="3" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="221">
@@ -3898,10 +4051,10 @@
         <v>216</v>
       </c>
       <c r="B221" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="C221" s="3" t="s">
         <v>398</v>
-      </c>
-      <c r="C221" s="3" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="222">
@@ -3909,10 +4062,10 @@
         <v>217</v>
       </c>
       <c r="B222" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="C222" s="3" t="s">
         <v>400</v>
-      </c>
-      <c r="C222" s="3" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="223">
@@ -3920,10 +4073,10 @@
         <v>218</v>
       </c>
       <c r="B223" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="C223" s="3" t="s">
         <v>402</v>
-      </c>
-      <c r="C223" s="3" t="s">
-        <v>403</v>
       </c>
     </row>
     <row r="224">
@@ -3931,10 +4084,10 @@
         <v>219</v>
       </c>
       <c r="B224" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="C224" s="3" t="s">
         <v>404</v>
-      </c>
-      <c r="C224" s="3" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="225">
@@ -3942,10 +4095,10 @@
         <v>220</v>
       </c>
       <c r="B225" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="C225" s="3" t="s">
         <v>406</v>
-      </c>
-      <c r="C225" s="3" t="s">
-        <v>407</v>
       </c>
     </row>
     <row r="226">
@@ -3953,10 +4106,10 @@
         <v>221</v>
       </c>
       <c r="B226" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="C226" s="3" t="s">
         <v>408</v>
-      </c>
-      <c r="C226" s="3" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="227">
@@ -3964,10 +4117,10 @@
         <v>222</v>
       </c>
       <c r="B227" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="C227" s="3" t="s">
         <v>410</v>
-      </c>
-      <c r="C227" s="3" t="s">
-        <v>411</v>
       </c>
     </row>
     <row r="228">
@@ -3975,10 +4128,10 @@
         <v>223</v>
       </c>
       <c r="B228" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="C228" s="3" t="s">
         <v>412</v>
-      </c>
-      <c r="C228" s="3" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="229">
@@ -3986,10 +4139,10 @@
         <v>224</v>
       </c>
       <c r="B229" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="C229" s="3" t="s">
         <v>414</v>
-      </c>
-      <c r="C229" s="3" t="s">
-        <v>415</v>
       </c>
     </row>
     <row r="230">
@@ -3997,10 +4150,10 @@
         <v>225</v>
       </c>
       <c r="B230" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="C230" s="3" t="s">
         <v>416</v>
-      </c>
-      <c r="C230" s="3" t="s">
-        <v>417</v>
       </c>
     </row>
     <row r="231">
@@ -4008,10 +4161,10 @@
         <v>226</v>
       </c>
       <c r="B231" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="C231" s="3" t="s">
         <v>418</v>
-      </c>
-      <c r="C231" s="3" t="s">
-        <v>419</v>
       </c>
     </row>
     <row r="232">
@@ -4019,10 +4172,10 @@
         <v>227</v>
       </c>
       <c r="B232" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="C232" s="3" t="s">
         <v>420</v>
-      </c>
-      <c r="C232" s="3" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="233">
@@ -4066,7 +4219,7 @@
         <v>427</v>
       </c>
       <c r="C236" s="3" t="s">
-        <v>428</v>
+        <v>255</v>
       </c>
     </row>
     <row r="237">
@@ -4074,10 +4227,10 @@
         <v>232</v>
       </c>
       <c r="B237" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="C237" s="3" t="s">
         <v>429</v>
-      </c>
-      <c r="C237" s="3" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="238">
@@ -4085,10 +4238,10 @@
         <v>233</v>
       </c>
       <c r="B238" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="C238" s="3" t="s">
         <v>431</v>
-      </c>
-      <c r="C238" s="3" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="239">
@@ -4132,7 +4285,7 @@
         <v>438</v>
       </c>
       <c r="C242" s="3" t="s">
-        <v>439</v>
+        <v>255</v>
       </c>
     </row>
     <row r="243">
@@ -4140,10 +4293,10 @@
         <v>238</v>
       </c>
       <c r="B243" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="C243" s="3" t="s">
         <v>440</v>
-      </c>
-      <c r="C243" s="3" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="244">
@@ -4151,10 +4304,10 @@
         <v>239</v>
       </c>
       <c r="B244" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="C244" s="3" t="s">
         <v>442</v>
-      </c>
-      <c r="C244" s="3" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="245">
@@ -4162,10 +4315,10 @@
         <v>240</v>
       </c>
       <c r="B245" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="C245" s="3" t="s">
         <v>444</v>
-      </c>
-      <c r="C245" s="3" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="246">
@@ -4173,10 +4326,10 @@
         <v>241</v>
       </c>
       <c r="B246" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="C246" s="3" t="s">
         <v>446</v>
-      </c>
-      <c r="C246" s="3" t="s">
-        <v>447</v>
       </c>
     </row>
     <row r="247">
@@ -4184,10 +4337,10 @@
         <v>242</v>
       </c>
       <c r="B247" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="C247" s="3" t="s">
         <v>448</v>
-      </c>
-      <c r="C247" s="3" t="s">
-        <v>449</v>
       </c>
     </row>
     <row r="248">
@@ -4195,10 +4348,10 @@
         <v>243</v>
       </c>
       <c r="B248" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="C248" s="3" t="s">
         <v>450</v>
-      </c>
-      <c r="C248" s="3" t="s">
-        <v>451</v>
       </c>
     </row>
     <row r="249">
@@ -4206,10 +4359,10 @@
         <v>244</v>
       </c>
       <c r="B249" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="C249" s="3" t="s">
         <v>452</v>
-      </c>
-      <c r="C249" s="3" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="250">
@@ -4217,10 +4370,10 @@
         <v>245</v>
       </c>
       <c r="B250" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="C250" s="3" t="s">
         <v>454</v>
-      </c>
-      <c r="C250" s="3" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="251">
@@ -4228,10 +4381,10 @@
         <v>246</v>
       </c>
       <c r="B251" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="C251" s="3" t="s">
         <v>456</v>
-      </c>
-      <c r="C251" s="3" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="252">
@@ -4239,10 +4392,10 @@
         <v>247</v>
       </c>
       <c r="B252" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="C252" s="3" t="s">
         <v>458</v>
-      </c>
-      <c r="C252" s="3" t="s">
-        <v>459</v>
       </c>
     </row>
     <row r="253">
@@ -4250,10 +4403,10 @@
         <v>248</v>
       </c>
       <c r="B253" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="C253" s="3" t="s">
         <v>460</v>
-      </c>
-      <c r="C253" s="3" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="254">
@@ -4261,10 +4414,10 @@
         <v>249</v>
       </c>
       <c r="B254" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="C254" s="3" t="s">
         <v>462</v>
-      </c>
-      <c r="C254" s="3" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="255">
@@ -4272,10 +4425,10 @@
         <v>250</v>
       </c>
       <c r="B255" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="C255" s="3" t="s">
         <v>464</v>
-      </c>
-      <c r="C255" s="3" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="256">
@@ -4308,7 +4461,7 @@
         <v>469</v>
       </c>
       <c r="C258" s="3" t="s">
-        <v>242</v>
+        <v>470</v>
       </c>
     </row>
     <row r="259">
@@ -4316,10 +4469,329 @@
         <v>254</v>
       </c>
       <c r="B259" s="3" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C259" s="3" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="3">
+        <v>255</v>
+      </c>
+      <c r="B260" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="C260" s="3" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="3">
+        <v>256</v>
+      </c>
+      <c r="B261" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="C261" s="3" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="3">
+        <v>257</v>
+      </c>
+      <c r="B262" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="C262" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="3">
+        <v>258</v>
+      </c>
+      <c r="B263" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="C263" s="3" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="3">
+        <v>259</v>
+      </c>
+      <c r="B264" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="C264" s="3" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="3">
+        <v>260</v>
+      </c>
+      <c r="B265" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C265" s="3" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="3">
+        <v>261</v>
+      </c>
+      <c r="B266" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="C266" s="3" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="3">
+        <v>262</v>
+      </c>
+      <c r="B267" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="C267" s="3" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="3">
+        <v>263</v>
+      </c>
+      <c r="B268" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="C268" s="3" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="3">
+        <v>264</v>
+      </c>
+      <c r="B269" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="C269" s="3" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="3">
         <v>265</v>
+      </c>
+      <c r="B270" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="C270" s="3" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="3">
+        <v>266</v>
+      </c>
+      <c r="B271" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="C271" s="3" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="3">
+        <v>267</v>
+      </c>
+      <c r="B272" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="C272" s="3" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="3">
+        <v>268</v>
+      </c>
+      <c r="B273" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="C273" s="3" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="3">
+        <v>269</v>
+      </c>
+      <c r="B274" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="C274" s="3" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="3">
+        <v>270</v>
+      </c>
+      <c r="B275" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="C275" s="3" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="3">
+        <v>271</v>
+      </c>
+      <c r="B276" s="3" t="s">
+        <v>500</v>
+      </c>
+      <c r="C276" s="3" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="3">
+        <v>272</v>
+      </c>
+      <c r="B277" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="C277" s="3" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="3">
+        <v>273</v>
+      </c>
+      <c r="B278" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="C278" s="3" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="3">
+        <v>274</v>
+      </c>
+      <c r="B279" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="C279" s="3" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="3">
+        <v>275</v>
+      </c>
+      <c r="B280" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="C280" s="3" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="3">
+        <v>276</v>
+      </c>
+      <c r="B281" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="C281" s="3" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="3">
+        <v>277</v>
+      </c>
+      <c r="B282" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="C282" s="3" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="3">
+        <v>278</v>
+      </c>
+      <c r="B283" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="C283" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="3">
+        <v>279</v>
+      </c>
+      <c r="B284" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="C284" s="3" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="3">
+        <v>280</v>
+      </c>
+      <c r="B285" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="C285" s="3" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="3">
+        <v>281</v>
+      </c>
+      <c r="B286" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="C286" s="3" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="3">
+        <v>282</v>
+      </c>
+      <c r="B287" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="C287" s="3" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="3">
+        <v>283</v>
+      </c>
+      <c r="B288" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="C288" s="3" t="s">
+        <v>521</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Update data Juni 2026, retrain forecast model, dan deploy ke HF Space (#20)
Update data Juni 2026 + retrain forecast model + deploy HF Space
</commit_message>
<xml_diff>
--- a/datasets/BI Rate (Data Inflasi)/Data Inflasi.xlsx
+++ b/datasets/BI Rate (Data Inflasi)/Data Inflasi.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="522">
   <si>
     <t>Data Inflasi</t>
   </si>
@@ -23,6 +23,30 @@
     <t>Periode</t>
   </si>
   <si>
+    <t>Juni 2026</t>
+  </si>
+  <si>
+    <t>3.34 %</t>
+  </si>
+  <si>
+    <t>Mei 2026</t>
+  </si>
+  <si>
+    <t>3.08 %</t>
+  </si>
+  <si>
+    <t>April 2026</t>
+  </si>
+  <si>
+    <t>2.42 %</t>
+  </si>
+  <si>
+    <t>Maret 2026</t>
+  </si>
+  <si>
+    <t>3.48 %</t>
+  </si>
+  <si>
     <t>Februari 2026</t>
   </si>
   <si>
@@ -209,9 +233,6 @@
     <t>Juli 2023</t>
   </si>
   <si>
-    <t>3.08 %</t>
-  </si>
-  <si>
     <t>Juni 2023</t>
   </si>
   <si>
@@ -1425,6 +1446,138 @@
   </si>
   <si>
     <t>Januari 2005</t>
+  </si>
+  <si>
+    <t>Desember 2004</t>
+  </si>
+  <si>
+    <t>6.4 %</t>
+  </si>
+  <si>
+    <t>November 2004</t>
+  </si>
+  <si>
+    <t>6.18 %</t>
+  </si>
+  <si>
+    <t>Oktober 2004</t>
+  </si>
+  <si>
+    <t>September 2004</t>
+  </si>
+  <si>
+    <t>6.27 %</t>
+  </si>
+  <si>
+    <t>Agustus 2004</t>
+  </si>
+  <si>
+    <t>6.67 %</t>
+  </si>
+  <si>
+    <t>Juli 2004</t>
+  </si>
+  <si>
+    <t>7.2 %</t>
+  </si>
+  <si>
+    <t>Juni 2004</t>
+  </si>
+  <si>
+    <t>Mei 2004</t>
+  </si>
+  <si>
+    <t>6.47 %</t>
+  </si>
+  <si>
+    <t>April 2004</t>
+  </si>
+  <si>
+    <t>5.92 %</t>
+  </si>
+  <si>
+    <t>Maret 2004</t>
+  </si>
+  <si>
+    <t>5.11 %</t>
+  </si>
+  <si>
+    <t>Februari 2004</t>
+  </si>
+  <si>
+    <t>4.6 %</t>
+  </si>
+  <si>
+    <t>Januari 2004</t>
+  </si>
+  <si>
+    <t>4.82 %</t>
+  </si>
+  <si>
+    <t>Desember 2003</t>
+  </si>
+  <si>
+    <t>5.16 %</t>
+  </si>
+  <si>
+    <t>November 2003</t>
+  </si>
+  <si>
+    <t>5.53 %</t>
+  </si>
+  <si>
+    <t>Oktober 2003</t>
+  </si>
+  <si>
+    <t>6.48 %</t>
+  </si>
+  <si>
+    <t>September 2003</t>
+  </si>
+  <si>
+    <t>Agustus 2003</t>
+  </si>
+  <si>
+    <t>Juli 2003</t>
+  </si>
+  <si>
+    <t>Juni 2003</t>
+  </si>
+  <si>
+    <t>6.98 %</t>
+  </si>
+  <si>
+    <t>Mei 2003</t>
+  </si>
+  <si>
+    <t>April 2003</t>
+  </si>
+  <si>
+    <t>7.62 %</t>
+  </si>
+  <si>
+    <t>Maret 2003</t>
+  </si>
+  <si>
+    <t>7.17 %</t>
+  </si>
+  <si>
+    <t>Februari 2003</t>
+  </si>
+  <si>
+    <t>7.6 %</t>
+  </si>
+  <si>
+    <t>Januari 2003</t>
+  </si>
+  <si>
+    <t>8.68 %</t>
+  </si>
+  <si>
+    <t>Desember 2002</t>
+  </si>
+  <si>
+    <t>0 %</t>
   </si>
 </sst>
 </file>
@@ -1500,7 +1653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="xr">
-  <dimension ref="A3:D259"/>
+  <dimension ref="A3:D288"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -1833,7 +1986,7 @@
         <v>57</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>12</v>
+        <v>58</v>
       </c>
     </row>
     <row r="34">
@@ -1841,10 +1994,10 @@
         <v>29</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35">
@@ -1852,10 +2005,10 @@
         <v>30</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36">
@@ -1863,10 +2016,10 @@
         <v>31</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37">
@@ -1874,10 +2027,10 @@
         <v>32</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38">
@@ -1921,7 +2074,7 @@
         <v>72</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>73</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42">
@@ -1929,10 +2082,10 @@
         <v>37</v>
       </c>
       <c r="B42" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C42" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="43">
@@ -1940,10 +2093,10 @@
         <v>38</v>
       </c>
       <c r="B43" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C43" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="44">
@@ -1951,10 +2104,10 @@
         <v>39</v>
       </c>
       <c r="B44" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C44" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="45">
@@ -1962,10 +2115,10 @@
         <v>40</v>
       </c>
       <c r="B45" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C45" s="3" t="s">
         <v>80</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="46">
@@ -1973,10 +2126,10 @@
         <v>41</v>
       </c>
       <c r="B46" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C46" s="3" t="s">
         <v>82</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="47">
@@ -1984,10 +2137,10 @@
         <v>42</v>
       </c>
       <c r="B47" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C47" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="48">
@@ -1995,10 +2148,10 @@
         <v>43</v>
       </c>
       <c r="B48" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C48" s="3" t="s">
         <v>86</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="49">
@@ -2006,10 +2159,10 @@
         <v>44</v>
       </c>
       <c r="B49" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C49" s="3" t="s">
         <v>88</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="50">
@@ -2017,10 +2170,10 @@
         <v>45</v>
       </c>
       <c r="B50" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C50" s="3" t="s">
         <v>90</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="51">
@@ -2028,10 +2181,10 @@
         <v>46</v>
       </c>
       <c r="B51" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C51" s="3" t="s">
         <v>92</v>
-      </c>
-      <c r="C51" s="3" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="52">
@@ -2075,7 +2228,7 @@
         <v>99</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>100</v>
+        <v>14</v>
       </c>
     </row>
     <row r="56">
@@ -2083,10 +2236,10 @@
         <v>51</v>
       </c>
       <c r="B56" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C56" s="3" t="s">
         <v>101</v>
-      </c>
-      <c r="C56" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="57">
@@ -2119,7 +2272,7 @@
         <v>106</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>22</v>
+        <v>107</v>
       </c>
     </row>
     <row r="60">
@@ -2127,10 +2280,10 @@
         <v>55</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>108</v>
+        <v>28</v>
       </c>
     </row>
     <row r="61">
@@ -2163,7 +2316,7 @@
         <v>113</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>114</v>
+        <v>30</v>
       </c>
     </row>
     <row r="64">
@@ -2171,10 +2324,10 @@
         <v>59</v>
       </c>
       <c r="B64" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C64" s="3" t="s">
         <v>115</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="65">
@@ -2182,10 +2335,10 @@
         <v>60</v>
       </c>
       <c r="B65" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C65" s="3" t="s">
         <v>117</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="66">
@@ -2193,10 +2346,10 @@
         <v>61</v>
       </c>
       <c r="B66" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C66" s="3" t="s">
         <v>119</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="67">
@@ -2204,10 +2357,10 @@
         <v>62</v>
       </c>
       <c r="B67" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C67" s="3" t="s">
         <v>121</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="68">
@@ -2218,7 +2371,7 @@
         <v>122</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
     <row r="69">
@@ -2226,10 +2379,10 @@
         <v>64</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
     </row>
     <row r="70">
@@ -2237,10 +2390,10 @@
         <v>65</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="71">
@@ -2248,10 +2401,10 @@
         <v>66</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>116</v>
+        <v>42</v>
       </c>
     </row>
     <row r="72">
@@ -2259,10 +2412,10 @@
         <v>67</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
     </row>
     <row r="73">
@@ -2270,10 +2423,10 @@
         <v>68</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
     </row>
     <row r="74">
@@ -2295,7 +2448,7 @@
         <v>133</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
     </row>
     <row r="76">
@@ -2303,10 +2456,10 @@
         <v>71</v>
       </c>
       <c r="B76" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C76" s="3" t="s">
         <v>135</v>
-      </c>
-      <c r="C76" s="3" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="77">
@@ -2314,10 +2467,10 @@
         <v>72</v>
       </c>
       <c r="B77" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C77" s="3" t="s">
         <v>137</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="78">
@@ -2325,10 +2478,10 @@
         <v>73</v>
       </c>
       <c r="B78" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C78" s="3" t="s">
         <v>139</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="79">
@@ -2336,10 +2489,10 @@
         <v>74</v>
       </c>
       <c r="B79" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C79" s="3" t="s">
         <v>141</v>
-      </c>
-      <c r="C79" s="3" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="80">
@@ -2347,10 +2500,10 @@
         <v>75</v>
       </c>
       <c r="B80" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C80" s="3" t="s">
         <v>143</v>
-      </c>
-      <c r="C80" s="3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="81">
@@ -2361,7 +2514,7 @@
         <v>144</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>48</v>
+        <v>145</v>
       </c>
     </row>
     <row r="82">
@@ -2369,10 +2522,10 @@
         <v>77</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="83">
@@ -2380,10 +2533,10 @@
         <v>78</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="84">
@@ -2391,10 +2544,10 @@
         <v>79</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>150</v>
+        <v>18</v>
       </c>
     </row>
     <row r="85">
@@ -2405,7 +2558,7 @@
         <v>151</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>152</v>
+        <v>56</v>
       </c>
     </row>
     <row r="86">
@@ -2413,10 +2566,10 @@
         <v>81</v>
       </c>
       <c r="B86" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C86" s="3" t="s">
         <v>153</v>
-      </c>
-      <c r="C86" s="3" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="87">
@@ -2424,10 +2577,10 @@
         <v>82</v>
       </c>
       <c r="B87" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C87" s="3" t="s">
         <v>155</v>
-      </c>
-      <c r="C87" s="3" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="88">
@@ -2460,7 +2613,7 @@
         <v>160</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>54</v>
+        <v>161</v>
       </c>
     </row>
     <row r="91">
@@ -2468,10 +2621,10 @@
         <v>86</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="92">
@@ -2482,7 +2635,7 @@
         <v>163</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>146</v>
+        <v>164</v>
       </c>
     </row>
     <row r="93">
@@ -2490,10 +2643,10 @@
         <v>88</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="94">
@@ -2501,10 +2654,10 @@
         <v>89</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>167</v>
+        <v>62</v>
       </c>
     </row>
     <row r="95">
@@ -2526,7 +2679,7 @@
         <v>170</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
     </row>
     <row r="97">
@@ -2534,10 +2687,10 @@
         <v>92</v>
       </c>
       <c r="B97" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C97" s="3" t="s">
         <v>172</v>
-      </c>
-      <c r="C97" s="3" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="98">
@@ -2545,10 +2698,10 @@
         <v>93</v>
       </c>
       <c r="B98" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="C98" s="3" t="s">
         <v>174</v>
-      </c>
-      <c r="C98" s="3" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="99">
@@ -2556,10 +2709,10 @@
         <v>94</v>
       </c>
       <c r="B99" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C99" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="C99" s="3" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="100">
@@ -2592,7 +2745,7 @@
         <v>181</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
     </row>
     <row r="103">
@@ -2600,10 +2753,10 @@
         <v>98</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
     </row>
     <row r="104">
@@ -2636,7 +2789,7 @@
         <v>188</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="107">
@@ -2644,10 +2797,10 @@
         <v>102</v>
       </c>
       <c r="B107" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C107" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="C107" s="3" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="108">
@@ -2655,10 +2808,10 @@
         <v>103</v>
       </c>
       <c r="B108" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="C108" s="3" t="s">
         <v>192</v>
-      </c>
-      <c r="C108" s="3" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="109">
@@ -2666,10 +2819,10 @@
         <v>104</v>
       </c>
       <c r="B109" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="C109" s="3" t="s">
         <v>194</v>
-      </c>
-      <c r="C109" s="3" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="110">
@@ -2677,10 +2830,10 @@
         <v>105</v>
       </c>
       <c r="B110" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="C110" s="3" t="s">
         <v>196</v>
-      </c>
-      <c r="C110" s="3" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="111">
@@ -2688,10 +2841,10 @@
         <v>106</v>
       </c>
       <c r="B111" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="C111" s="3" t="s">
         <v>198</v>
-      </c>
-      <c r="C111" s="3" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="112">
@@ -2713,7 +2866,7 @@
         <v>201</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>185</v>
+        <v>202</v>
       </c>
     </row>
     <row r="114">
@@ -2721,10 +2874,10 @@
         <v>109</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="115">
@@ -2732,10 +2885,10 @@
         <v>110</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>150</v>
+        <v>78</v>
       </c>
     </row>
     <row r="116">
@@ -2743,10 +2896,10 @@
         <v>111</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="117">
@@ -2754,10 +2907,10 @@
         <v>112</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="118">
@@ -2765,10 +2918,10 @@
         <v>113</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="119">
@@ -2776,10 +2929,10 @@
         <v>114</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>211</v>
+        <v>157</v>
       </c>
     </row>
     <row r="120">
@@ -2801,7 +2954,7 @@
         <v>214</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>215</v>
+        <v>196</v>
       </c>
     </row>
     <row r="122">
@@ -2809,10 +2962,10 @@
         <v>117</v>
       </c>
       <c r="B122" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="C122" s="3" t="s">
         <v>216</v>
-      </c>
-      <c r="C122" s="3" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="123">
@@ -2820,10 +2973,10 @@
         <v>118</v>
       </c>
       <c r="B123" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="C123" s="3" t="s">
         <v>218</v>
-      </c>
-      <c r="C123" s="3" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="124">
@@ -2831,10 +2984,10 @@
         <v>119</v>
       </c>
       <c r="B124" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="C124" s="3" t="s">
         <v>220</v>
-      </c>
-      <c r="C124" s="3" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="125">
@@ -2842,10 +2995,10 @@
         <v>120</v>
       </c>
       <c r="B125" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="C125" s="3" t="s">
         <v>222</v>
-      </c>
-      <c r="C125" s="3" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="126">
@@ -2853,10 +3006,10 @@
         <v>121</v>
       </c>
       <c r="B126" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="C126" s="3" t="s">
         <v>224</v>
-      </c>
-      <c r="C126" s="3" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="127">
@@ -2864,10 +3017,10 @@
         <v>122</v>
       </c>
       <c r="B127" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C127" s="3" t="s">
         <v>226</v>
-      </c>
-      <c r="C127" s="3" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="128">
@@ -2875,10 +3028,10 @@
         <v>123</v>
       </c>
       <c r="B128" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="C128" s="3" t="s">
         <v>228</v>
-      </c>
-      <c r="C128" s="3" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="129">
@@ -2886,10 +3039,10 @@
         <v>124</v>
       </c>
       <c r="B129" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="C129" s="3" t="s">
         <v>230</v>
-      </c>
-      <c r="C129" s="3" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="130">
@@ -2897,10 +3050,10 @@
         <v>125</v>
       </c>
       <c r="B130" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="C130" s="3" t="s">
         <v>232</v>
-      </c>
-      <c r="C130" s="3" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="131">
@@ -2908,10 +3061,10 @@
         <v>126</v>
       </c>
       <c r="B131" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C131" s="3" t="s">
         <v>234</v>
-      </c>
-      <c r="C131" s="3" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="132">
@@ -2919,10 +3072,10 @@
         <v>127</v>
       </c>
       <c r="B132" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="C132" s="3" t="s">
         <v>236</v>
-      </c>
-      <c r="C132" s="3" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="133">
@@ -2930,10 +3083,10 @@
         <v>128</v>
       </c>
       <c r="B133" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="C133" s="3" t="s">
         <v>238</v>
-      </c>
-      <c r="C133" s="3" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="134">
@@ -2941,10 +3094,10 @@
         <v>129</v>
       </c>
       <c r="B134" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C134" s="3" t="s">
         <v>240</v>
-      </c>
-      <c r="C134" s="3" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="135">
@@ -2988,7 +3141,7 @@
         <v>247</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="139">
@@ -2996,10 +3149,10 @@
         <v>134</v>
       </c>
       <c r="B139" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="C139" s="3" t="s">
         <v>249</v>
-      </c>
-      <c r="C139" s="3" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="140">
@@ -3007,10 +3160,10 @@
         <v>135</v>
       </c>
       <c r="B140" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="C140" s="3" t="s">
         <v>251</v>
-      </c>
-      <c r="C140" s="3" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="141">
@@ -3018,10 +3171,10 @@
         <v>136</v>
       </c>
       <c r="B141" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="C141" s="3" t="s">
         <v>253</v>
-      </c>
-      <c r="C141" s="3" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="142">
@@ -3029,10 +3182,10 @@
         <v>137</v>
       </c>
       <c r="B142" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="C142" s="3" t="s">
         <v>255</v>
-      </c>
-      <c r="C142" s="3" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="143">
@@ -3040,10 +3193,10 @@
         <v>138</v>
       </c>
       <c r="B143" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="C143" s="3" t="s">
         <v>257</v>
-      </c>
-      <c r="C143" s="3" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="144">
@@ -3051,10 +3204,10 @@
         <v>139</v>
       </c>
       <c r="B144" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="C144" s="3" t="s">
         <v>259</v>
-      </c>
-      <c r="C144" s="3" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="145">
@@ -3062,10 +3215,10 @@
         <v>140</v>
       </c>
       <c r="B145" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="C145" s="3" t="s">
         <v>261</v>
-      </c>
-      <c r="C145" s="3" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="146">
@@ -3153,7 +3306,7 @@
         <v>275</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
     </row>
     <row r="154">
@@ -3161,10 +3314,10 @@
         <v>149</v>
       </c>
       <c r="B154" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="C154" s="3" t="s">
         <v>277</v>
-      </c>
-      <c r="C154" s="3" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="155">
@@ -3172,10 +3325,10 @@
         <v>150</v>
       </c>
       <c r="B155" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="C155" s="3" t="s">
         <v>279</v>
-      </c>
-      <c r="C155" s="3" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="156">
@@ -3183,10 +3336,10 @@
         <v>151</v>
       </c>
       <c r="B156" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="C156" s="3" t="s">
         <v>281</v>
-      </c>
-      <c r="C156" s="3" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="157">
@@ -3194,10 +3347,10 @@
         <v>152</v>
       </c>
       <c r="B157" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="C157" s="3" t="s">
         <v>283</v>
-      </c>
-      <c r="C157" s="3" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="158">
@@ -3205,10 +3358,10 @@
         <v>153</v>
       </c>
       <c r="B158" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="C158" s="3" t="s">
         <v>285</v>
-      </c>
-      <c r="C158" s="3" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="159">
@@ -3216,10 +3369,10 @@
         <v>154</v>
       </c>
       <c r="B159" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="C159" s="3" t="s">
         <v>287</v>
-      </c>
-      <c r="C159" s="3" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="160">
@@ -3241,7 +3394,7 @@
         <v>290</v>
       </c>
       <c r="C161" s="3" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
     </row>
     <row r="162">
@@ -3249,10 +3402,10 @@
         <v>157</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C162" s="3" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="163">
@@ -3260,10 +3413,10 @@
         <v>158</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C163" s="3" t="s">
-        <v>294</v>
+        <v>82</v>
       </c>
     </row>
     <row r="164">
@@ -3285,7 +3438,7 @@
         <v>297</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
     </row>
     <row r="166">
@@ -3293,10 +3446,10 @@
         <v>161</v>
       </c>
       <c r="B166" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="C166" s="3" t="s">
         <v>299</v>
-      </c>
-      <c r="C166" s="3" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="167">
@@ -3304,10 +3457,10 @@
         <v>162</v>
       </c>
       <c r="B167" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="C167" s="3" t="s">
         <v>301</v>
-      </c>
-      <c r="C167" s="3" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="168">
@@ -3315,10 +3468,10 @@
         <v>163</v>
       </c>
       <c r="B168" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="C168" s="3" t="s">
         <v>303</v>
-      </c>
-      <c r="C168" s="3" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="169">
@@ -3326,10 +3479,10 @@
         <v>164</v>
       </c>
       <c r="B169" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="C169" s="3" t="s">
         <v>305</v>
-      </c>
-      <c r="C169" s="3" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="170">
@@ -3337,10 +3490,10 @@
         <v>165</v>
       </c>
       <c r="B170" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="C170" s="3" t="s">
         <v>307</v>
-      </c>
-      <c r="C170" s="3" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="171">
@@ -3351,7 +3504,7 @@
         <v>308</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>223</v>
+        <v>309</v>
       </c>
     </row>
     <row r="172">
@@ -3359,10 +3512,10 @@
         <v>167</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C172" s="3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="173">
@@ -3370,10 +3523,10 @@
         <v>168</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C173" s="3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="174">
@@ -3381,10 +3534,10 @@
         <v>169</v>
       </c>
       <c r="B174" s="3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C174" s="3" t="s">
-        <v>314</v>
+        <v>265</v>
       </c>
     </row>
     <row r="175">
@@ -3395,7 +3548,7 @@
         <v>315</v>
       </c>
       <c r="C175" s="3" t="s">
-        <v>316</v>
+        <v>230</v>
       </c>
     </row>
     <row r="176">
@@ -3403,10 +3556,10 @@
         <v>171</v>
       </c>
       <c r="B176" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="C176" s="3" t="s">
         <v>317</v>
-      </c>
-      <c r="C176" s="3" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="177">
@@ -3414,10 +3567,10 @@
         <v>172</v>
       </c>
       <c r="B177" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="C177" s="3" t="s">
         <v>319</v>
-      </c>
-      <c r="C177" s="3" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="178">
@@ -3425,10 +3578,10 @@
         <v>173</v>
       </c>
       <c r="B178" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="C178" s="3" t="s">
         <v>321</v>
-      </c>
-      <c r="C178" s="3" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="179">
@@ -3439,7 +3592,7 @@
         <v>322</v>
       </c>
       <c r="C179" s="3" t="s">
-        <v>300</v>
+        <v>323</v>
       </c>
     </row>
     <row r="180">
@@ -3447,10 +3600,10 @@
         <v>175</v>
       </c>
       <c r="B180" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C180" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="181">
@@ -3458,10 +3611,10 @@
         <v>176</v>
       </c>
       <c r="B181" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C181" s="3" t="s">
-        <v>300</v>
+        <v>327</v>
       </c>
     </row>
     <row r="182">
@@ -3469,10 +3622,10 @@
         <v>177</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C182" s="3" t="s">
-        <v>327</v>
+        <v>232</v>
       </c>
     </row>
     <row r="183">
@@ -3480,10 +3633,10 @@
         <v>178</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C183" s="3" t="s">
-        <v>329</v>
+        <v>307</v>
       </c>
     </row>
     <row r="184">
@@ -3505,7 +3658,7 @@
         <v>332</v>
       </c>
       <c r="C185" s="3" t="s">
-        <v>333</v>
+        <v>307</v>
       </c>
     </row>
     <row r="186">
@@ -3513,10 +3666,10 @@
         <v>181</v>
       </c>
       <c r="B186" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C186" s="3" t="s">
         <v>334</v>
-      </c>
-      <c r="C186" s="3" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="187">
@@ -3524,10 +3677,10 @@
         <v>182</v>
       </c>
       <c r="B187" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="C187" s="3" t="s">
         <v>336</v>
-      </c>
-      <c r="C187" s="3" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="188">
@@ -3535,10 +3688,10 @@
         <v>183</v>
       </c>
       <c r="B188" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="C188" s="3" t="s">
         <v>338</v>
-      </c>
-      <c r="C188" s="3" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="189">
@@ -3582,7 +3735,7 @@
         <v>345</v>
       </c>
       <c r="C192" s="3" t="s">
-        <v>346</v>
+        <v>257</v>
       </c>
     </row>
     <row r="193">
@@ -3590,10 +3743,10 @@
         <v>188</v>
       </c>
       <c r="B193" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="C193" s="3" t="s">
         <v>347</v>
-      </c>
-      <c r="C193" s="3" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="194">
@@ -3601,10 +3754,10 @@
         <v>189</v>
       </c>
       <c r="B194" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="C194" s="3" t="s">
         <v>349</v>
-      </c>
-      <c r="C194" s="3" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="195">
@@ -3612,10 +3765,10 @@
         <v>190</v>
       </c>
       <c r="B195" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="C195" s="3" t="s">
         <v>351</v>
-      </c>
-      <c r="C195" s="3" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="196">
@@ -3623,10 +3776,10 @@
         <v>191</v>
       </c>
       <c r="B196" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="C196" s="3" t="s">
         <v>353</v>
-      </c>
-      <c r="C196" s="3" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="197">
@@ -3634,10 +3787,10 @@
         <v>192</v>
       </c>
       <c r="B197" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="C197" s="3" t="s">
         <v>355</v>
-      </c>
-      <c r="C197" s="3" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="198">
@@ -3645,10 +3798,10 @@
         <v>193</v>
       </c>
       <c r="B198" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="C198" s="3" t="s">
         <v>357</v>
-      </c>
-      <c r="C198" s="3" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="199">
@@ -3656,10 +3809,10 @@
         <v>194</v>
       </c>
       <c r="B199" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="C199" s="3" t="s">
         <v>359</v>
-      </c>
-      <c r="C199" s="3" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="200">
@@ -3692,7 +3845,7 @@
         <v>364</v>
       </c>
       <c r="C202" s="3" t="s">
-        <v>54</v>
+        <v>365</v>
       </c>
     </row>
     <row r="203">
@@ -3700,10 +3853,10 @@
         <v>198</v>
       </c>
       <c r="B203" s="3" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C203" s="3" t="s">
-        <v>157</v>
+        <v>198</v>
       </c>
     </row>
     <row r="204">
@@ -3711,10 +3864,10 @@
         <v>199</v>
       </c>
       <c r="B204" s="3" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C204" s="3" t="s">
-        <v>52</v>
+        <v>368</v>
       </c>
     </row>
     <row r="205">
@@ -3722,10 +3875,10 @@
         <v>200</v>
       </c>
       <c r="B205" s="3" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C205" s="3" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="206">
@@ -3733,10 +3886,10 @@
         <v>201</v>
       </c>
       <c r="B206" s="3" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C206" s="3" t="s">
-        <v>316</v>
+        <v>62</v>
       </c>
     </row>
     <row r="207">
@@ -3744,10 +3897,10 @@
         <v>202</v>
       </c>
       <c r="B207" s="3" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="C207" s="3" t="s">
-        <v>371</v>
+        <v>164</v>
       </c>
     </row>
     <row r="208">
@@ -3755,10 +3908,10 @@
         <v>203</v>
       </c>
       <c r="B208" s="3" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C208" s="3" t="s">
-        <v>373</v>
+        <v>60</v>
       </c>
     </row>
     <row r="209">
@@ -3780,7 +3933,7 @@
         <v>376</v>
       </c>
       <c r="C210" s="3" t="s">
-        <v>377</v>
+        <v>323</v>
       </c>
     </row>
     <row r="211">
@@ -3788,10 +3941,10 @@
         <v>206</v>
       </c>
       <c r="B211" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="C211" s="3" t="s">
         <v>378</v>
-      </c>
-      <c r="C211" s="3" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="212">
@@ -3799,10 +3952,10 @@
         <v>207</v>
       </c>
       <c r="B212" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="C212" s="3" t="s">
         <v>380</v>
-      </c>
-      <c r="C212" s="3" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="213">
@@ -3810,10 +3963,10 @@
         <v>208</v>
       </c>
       <c r="B213" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="C213" s="3" t="s">
         <v>382</v>
-      </c>
-      <c r="C213" s="3" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="214">
@@ -3821,10 +3974,10 @@
         <v>209</v>
       </c>
       <c r="B214" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="C214" s="3" t="s">
         <v>384</v>
-      </c>
-      <c r="C214" s="3" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="215">
@@ -3832,10 +3985,10 @@
         <v>210</v>
       </c>
       <c r="B215" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="C215" s="3" t="s">
         <v>386</v>
-      </c>
-      <c r="C215" s="3" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="216">
@@ -3843,10 +3996,10 @@
         <v>211</v>
       </c>
       <c r="B216" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="C216" s="3" t="s">
         <v>388</v>
-      </c>
-      <c r="C216" s="3" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="217">
@@ -3854,10 +4007,10 @@
         <v>212</v>
       </c>
       <c r="B217" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C217" s="3" t="s">
         <v>390</v>
-      </c>
-      <c r="C217" s="3" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="218">
@@ -3865,10 +4018,10 @@
         <v>213</v>
       </c>
       <c r="B218" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="C218" s="3" t="s">
         <v>392</v>
-      </c>
-      <c r="C218" s="3" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="219">
@@ -3876,10 +4029,10 @@
         <v>214</v>
       </c>
       <c r="B219" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C219" s="3" t="s">
         <v>394</v>
-      </c>
-      <c r="C219" s="3" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="220">
@@ -3887,10 +4040,10 @@
         <v>215</v>
       </c>
       <c r="B220" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="C220" s="3" t="s">
         <v>396</v>
-      </c>
-      <c r="C220" s="3" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="221">
@@ -3898,10 +4051,10 @@
         <v>216</v>
       </c>
       <c r="B221" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="C221" s="3" t="s">
         <v>398</v>
-      </c>
-      <c r="C221" s="3" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="222">
@@ -3909,10 +4062,10 @@
         <v>217</v>
       </c>
       <c r="B222" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="C222" s="3" t="s">
         <v>400</v>
-      </c>
-      <c r="C222" s="3" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="223">
@@ -3920,10 +4073,10 @@
         <v>218</v>
       </c>
       <c r="B223" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="C223" s="3" t="s">
         <v>402</v>
-      </c>
-      <c r="C223" s="3" t="s">
-        <v>403</v>
       </c>
     </row>
     <row r="224">
@@ -3931,10 +4084,10 @@
         <v>219</v>
       </c>
       <c r="B224" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="C224" s="3" t="s">
         <v>404</v>
-      </c>
-      <c r="C224" s="3" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="225">
@@ -3942,10 +4095,10 @@
         <v>220</v>
       </c>
       <c r="B225" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="C225" s="3" t="s">
         <v>406</v>
-      </c>
-      <c r="C225" s="3" t="s">
-        <v>407</v>
       </c>
     </row>
     <row r="226">
@@ -3953,10 +4106,10 @@
         <v>221</v>
       </c>
       <c r="B226" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="C226" s="3" t="s">
         <v>408</v>
-      </c>
-      <c r="C226" s="3" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="227">
@@ -3964,10 +4117,10 @@
         <v>222</v>
       </c>
       <c r="B227" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="C227" s="3" t="s">
         <v>410</v>
-      </c>
-      <c r="C227" s="3" t="s">
-        <v>411</v>
       </c>
     </row>
     <row r="228">
@@ -3975,10 +4128,10 @@
         <v>223</v>
       </c>
       <c r="B228" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="C228" s="3" t="s">
         <v>412</v>
-      </c>
-      <c r="C228" s="3" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="229">
@@ -3986,10 +4139,10 @@
         <v>224</v>
       </c>
       <c r="B229" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="C229" s="3" t="s">
         <v>414</v>
-      </c>
-      <c r="C229" s="3" t="s">
-        <v>415</v>
       </c>
     </row>
     <row r="230">
@@ -3997,10 +4150,10 @@
         <v>225</v>
       </c>
       <c r="B230" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="C230" s="3" t="s">
         <v>416</v>
-      </c>
-      <c r="C230" s="3" t="s">
-        <v>417</v>
       </c>
     </row>
     <row r="231">
@@ -4008,10 +4161,10 @@
         <v>226</v>
       </c>
       <c r="B231" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="C231" s="3" t="s">
         <v>418</v>
-      </c>
-      <c r="C231" s="3" t="s">
-        <v>419</v>
       </c>
     </row>
     <row r="232">
@@ -4019,10 +4172,10 @@
         <v>227</v>
       </c>
       <c r="B232" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="C232" s="3" t="s">
         <v>420</v>
-      </c>
-      <c r="C232" s="3" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="233">
@@ -4066,7 +4219,7 @@
         <v>427</v>
       </c>
       <c r="C236" s="3" t="s">
-        <v>428</v>
+        <v>255</v>
       </c>
     </row>
     <row r="237">
@@ -4074,10 +4227,10 @@
         <v>232</v>
       </c>
       <c r="B237" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="C237" s="3" t="s">
         <v>429</v>
-      </c>
-      <c r="C237" s="3" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="238">
@@ -4085,10 +4238,10 @@
         <v>233</v>
       </c>
       <c r="B238" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="C238" s="3" t="s">
         <v>431</v>
-      </c>
-      <c r="C238" s="3" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="239">
@@ -4132,7 +4285,7 @@
         <v>438</v>
       </c>
       <c r="C242" s="3" t="s">
-        <v>439</v>
+        <v>255</v>
       </c>
     </row>
     <row r="243">
@@ -4140,10 +4293,10 @@
         <v>238</v>
       </c>
       <c r="B243" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="C243" s="3" t="s">
         <v>440</v>
-      </c>
-      <c r="C243" s="3" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="244">
@@ -4151,10 +4304,10 @@
         <v>239</v>
       </c>
       <c r="B244" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="C244" s="3" t="s">
         <v>442</v>
-      </c>
-      <c r="C244" s="3" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="245">
@@ -4162,10 +4315,10 @@
         <v>240</v>
       </c>
       <c r="B245" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="C245" s="3" t="s">
         <v>444</v>
-      </c>
-      <c r="C245" s="3" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="246">
@@ -4173,10 +4326,10 @@
         <v>241</v>
       </c>
       <c r="B246" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="C246" s="3" t="s">
         <v>446</v>
-      </c>
-      <c r="C246" s="3" t="s">
-        <v>447</v>
       </c>
     </row>
     <row r="247">
@@ -4184,10 +4337,10 @@
         <v>242</v>
       </c>
       <c r="B247" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="C247" s="3" t="s">
         <v>448</v>
-      </c>
-      <c r="C247" s="3" t="s">
-        <v>449</v>
       </c>
     </row>
     <row r="248">
@@ -4195,10 +4348,10 @@
         <v>243</v>
       </c>
       <c r="B248" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="C248" s="3" t="s">
         <v>450</v>
-      </c>
-      <c r="C248" s="3" t="s">
-        <v>451</v>
       </c>
     </row>
     <row r="249">
@@ -4206,10 +4359,10 @@
         <v>244</v>
       </c>
       <c r="B249" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="C249" s="3" t="s">
         <v>452</v>
-      </c>
-      <c r="C249" s="3" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="250">
@@ -4217,10 +4370,10 @@
         <v>245</v>
       </c>
       <c r="B250" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="C250" s="3" t="s">
         <v>454</v>
-      </c>
-      <c r="C250" s="3" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="251">
@@ -4228,10 +4381,10 @@
         <v>246</v>
       </c>
       <c r="B251" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="C251" s="3" t="s">
         <v>456</v>
-      </c>
-      <c r="C251" s="3" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="252">
@@ -4239,10 +4392,10 @@
         <v>247</v>
       </c>
       <c r="B252" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="C252" s="3" t="s">
         <v>458</v>
-      </c>
-      <c r="C252" s="3" t="s">
-        <v>459</v>
       </c>
     </row>
     <row r="253">
@@ -4250,10 +4403,10 @@
         <v>248</v>
       </c>
       <c r="B253" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="C253" s="3" t="s">
         <v>460</v>
-      </c>
-      <c r="C253" s="3" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="254">
@@ -4261,10 +4414,10 @@
         <v>249</v>
       </c>
       <c r="B254" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="C254" s="3" t="s">
         <v>462</v>
-      </c>
-      <c r="C254" s="3" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="255">
@@ -4272,10 +4425,10 @@
         <v>250</v>
       </c>
       <c r="B255" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="C255" s="3" t="s">
         <v>464</v>
-      </c>
-      <c r="C255" s="3" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="256">
@@ -4308,7 +4461,7 @@
         <v>469</v>
       </c>
       <c r="C258" s="3" t="s">
-        <v>242</v>
+        <v>470</v>
       </c>
     </row>
     <row r="259">
@@ -4316,10 +4469,329 @@
         <v>254</v>
       </c>
       <c r="B259" s="3" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C259" s="3" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="3">
+        <v>255</v>
+      </c>
+      <c r="B260" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="C260" s="3" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="3">
+        <v>256</v>
+      </c>
+      <c r="B261" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="C261" s="3" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="3">
+        <v>257</v>
+      </c>
+      <c r="B262" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="C262" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="3">
+        <v>258</v>
+      </c>
+      <c r="B263" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="C263" s="3" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="3">
+        <v>259</v>
+      </c>
+      <c r="B264" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="C264" s="3" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="3">
+        <v>260</v>
+      </c>
+      <c r="B265" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C265" s="3" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="3">
+        <v>261</v>
+      </c>
+      <c r="B266" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="C266" s="3" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="3">
+        <v>262</v>
+      </c>
+      <c r="B267" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="C267" s="3" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="3">
+        <v>263</v>
+      </c>
+      <c r="B268" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="C268" s="3" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="3">
+        <v>264</v>
+      </c>
+      <c r="B269" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="C269" s="3" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="3">
         <v>265</v>
+      </c>
+      <c r="B270" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="C270" s="3" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="3">
+        <v>266</v>
+      </c>
+      <c r="B271" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="C271" s="3" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="3">
+        <v>267</v>
+      </c>
+      <c r="B272" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="C272" s="3" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="3">
+        <v>268</v>
+      </c>
+      <c r="B273" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="C273" s="3" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="3">
+        <v>269</v>
+      </c>
+      <c r="B274" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="C274" s="3" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="3">
+        <v>270</v>
+      </c>
+      <c r="B275" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="C275" s="3" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="3">
+        <v>271</v>
+      </c>
+      <c r="B276" s="3" t="s">
+        <v>500</v>
+      </c>
+      <c r="C276" s="3" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="3">
+        <v>272</v>
+      </c>
+      <c r="B277" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="C277" s="3" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="3">
+        <v>273</v>
+      </c>
+      <c r="B278" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="C278" s="3" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="3">
+        <v>274</v>
+      </c>
+      <c r="B279" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="C279" s="3" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="3">
+        <v>275</v>
+      </c>
+      <c r="B280" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="C280" s="3" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="3">
+        <v>276</v>
+      </c>
+      <c r="B281" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="C281" s="3" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="3">
+        <v>277</v>
+      </c>
+      <c r="B282" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="C282" s="3" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="3">
+        <v>278</v>
+      </c>
+      <c r="B283" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="C283" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="3">
+        <v>279</v>
+      </c>
+      <c r="B284" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="C284" s="3" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="3">
+        <v>280</v>
+      </c>
+      <c r="B285" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="C285" s="3" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="3">
+        <v>281</v>
+      </c>
+      <c r="B286" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="C286" s="3" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="3">
+        <v>282</v>
+      </c>
+      <c r="B287" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="C287" s="3" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="3">
+        <v>283</v>
+      </c>
+      <c r="B288" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="C288" s="3" t="s">
+        <v>521</v>
       </c>
     </row>
   </sheetData>

</xml_diff>